<commit_message>
working :) I hate everyone.
</commit_message>
<xml_diff>
--- a/sample.xlsx
+++ b/sample.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="60" uniqueCount="57">
   <si>
     <t>id</t>
   </si>
@@ -46,9 +46,6 @@
     <t>updated_at</t>
   </si>
   <si>
-    <t>is_active</t>
-  </si>
-  <si>
     <t>John</t>
   </si>
   <si>
@@ -64,9 +61,6 @@
     <t>Engineering</t>
   </si>
   <si>
-    <t>true</t>
-  </si>
-  <si>
     <t>Jane</t>
   </si>
   <si>
@@ -80,9 +74,6 @@
   </si>
   <si>
     <t>HR</t>
-  </si>
-  <si>
-    <t>false</t>
   </si>
   <si>
     <t>Robert</t>
@@ -253,7 +244,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0"/>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="1" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -279,20 +270,17 @@
     <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf xfId="0" numFmtId="0" borderId="1" applyBorder="1" fontId="2" applyFont="1" fillId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf xfId="0" numFmtId="3" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
     <xf xfId="0" numFmtId="0" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="164" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
     <xf xfId="0" numFmtId="165" applyNumberFormat="1" borderId="0" fontId="0" fillId="0" applyAlignment="1">
-      <alignment horizontal="general"/>
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -596,20 +584,19 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:K11"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="2" max="2" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="3" max="3" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="4" max="4" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="5" max="5" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="6" max="6" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="7" max="7" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="8" max="8" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="9" max="9" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="10" max="10" style="13" width="13.576428571428572" customWidth="1" bestFit="1"/>
-    <col min="11" max="11" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="1" max="1" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="2" max="2" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="3" max="3" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="4" max="4" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="5" max="5" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="6" max="6" style="10" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="7" max="7" style="9" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="8" max="8" style="11" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="9" max="9" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
+    <col min="10" max="10" style="12" width="13.576428571428572" customWidth="1" bestFit="1"/>
   </cols>
   <sheetData>
     <row x14ac:dyDescent="0.25" r="1" customHeight="1" ht="18.75">
@@ -643,28 +630,25 @@
       <c r="J1" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>10</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="2" customHeight="1" ht="18.75">
       <c r="A2" s="5">
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="E2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="F2" s="6" t="s">
         <v>14</v>
-      </c>
-      <c r="F2" s="6" t="s">
-        <v>15</v>
       </c>
       <c r="G2" s="5">
         <v>65000</v>
@@ -677,9 +661,6 @@
       </c>
       <c r="J2" s="8">
         <v>45745.5</v>
-      </c>
-      <c r="K2" s="9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="18.75">
@@ -687,19 +668,19 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="E3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="F3" s="6" t="s">
         <v>19</v>
-      </c>
-      <c r="E3" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="F3" s="6" t="s">
-        <v>21</v>
       </c>
       <c r="G3" s="5">
         <v>55000</v>
@@ -712,9 +693,6 @@
       </c>
       <c r="J3" s="8">
         <v>45745.40972222222</v>
-      </c>
-      <c r="K3" s="9" t="s">
-        <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="18.75">
@@ -722,19 +700,19 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="6" t="s">
+      <c r="F4" s="6" t="s">
         <v>24</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>27</v>
       </c>
       <c r="G4" s="5">
         <v>72000</v>
@@ -747,9 +725,6 @@
       </c>
       <c r="J4" s="8">
         <v>45745.461805555555</v>
-      </c>
-      <c r="K4" s="9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="18.75">
@@ -757,19 +732,19 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>30</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="6" t="s">
-        <v>32</v>
       </c>
       <c r="G5" s="5">
         <v>68000</v>
@@ -782,9 +757,6 @@
       </c>
       <c r="J5" s="8">
         <v>45745.48263888889</v>
-      </c>
-      <c r="K5" s="9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="6" customHeight="1" ht="18.75">
@@ -792,19 +764,19 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="C6" s="6" t="s">
+      <c r="F6" s="6" t="s">
         <v>34</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F6" s="6" t="s">
-        <v>37</v>
       </c>
       <c r="G6" s="5">
         <v>80000</v>
@@ -817,9 +789,6 @@
       </c>
       <c r="J6" s="8">
         <v>45745.427083333336</v>
-      </c>
-      <c r="K6" s="9" t="s">
-        <v>22</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="18.75">
@@ -827,19 +796,19 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>37</v>
+      </c>
+      <c r="E7" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C7" s="6" t="s">
+      <c r="F7" s="6" t="s">
         <v>39</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>42</v>
       </c>
       <c r="G7" s="5">
         <v>75000</v>
@@ -852,9 +821,6 @@
       </c>
       <c r="J7" s="8">
         <v>45745.399305555555</v>
-      </c>
-      <c r="K7" s="9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="18.75">
@@ -862,19 +828,19 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E8" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="C8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>44</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>46</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>47</v>
       </c>
       <c r="G8" s="5">
         <v>60000</v>
@@ -887,9 +853,6 @@
       </c>
       <c r="J8" s="8">
         <v>45745.51388888889</v>
-      </c>
-      <c r="K8" s="9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="18.75">
@@ -897,19 +860,19 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="E9" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>49</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>50</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>51</v>
-      </c>
       <c r="F9" s="6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G9" s="5">
         <v>70000</v>
@@ -922,9 +885,6 @@
       </c>
       <c r="J9" s="8">
         <v>45745.45138888889</v>
-      </c>
-      <c r="K9" s="9" t="s">
-        <v>16</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="18.75">
@@ -932,19 +892,19 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>53</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>55</v>
-      </c>
       <c r="F10" s="6" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="G10" s="5">
         <v>53000</v>
@@ -958,28 +918,25 @@
       <c r="J10" s="8">
         <v>45745.37847222222</v>
       </c>
-      <c r="K10" s="9" t="s">
-        <v>16</v>
-      </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="18.75">
       <c r="A11" s="5">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B11" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>58</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>59</v>
-      </c>
       <c r="F11" s="6" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="G11" s="5">
         <v>72000</v>
@@ -988,13 +945,10 @@
         <v>44464</v>
       </c>
       <c r="I11" s="8">
-        <v>45745.520833333336</v>
+        <v>45745.020833333336</v>
       </c>
       <c r="J11" s="8">
-        <v>45745.524305555555</v>
-      </c>
-      <c r="K11" s="9" t="s">
-        <v>22</v>
+        <v>45745.024305555555</v>
       </c>
     </row>
   </sheetData>

</xml_diff>